<commit_message>
updated the whole pipeline to follow the new idea of using the proportions instead of the PCs. updated also the fine mapping
</commit_message>
<xml_diff>
--- a/tables_plots/table_hits_wind.xlsx
+++ b/tables_plots/table_hits_wind.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,12 +441,12 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>ancestry tested</t>
+          <t>Ancestry</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>OR (CI = 95%)</t>
+          <t>OR (CI 95%)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -456,228 +456,274 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>lambda_GC</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>chr</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>START</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>END</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>chr</t>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>n_sig_windows</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HC221_Diabetes</t>
+          <t>HC1574_AD_myocardial_infarction</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10q25.3</t>
+          <t>5q14.3</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>WAS</t>
+          <t>AFR</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.66588 - (1.41207, 1.96531)</t>
+          <t>0.532905 (0.418964, 0.677832)</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>1.43519e-09</v>
+        <v>2.92534e-07</v>
       </c>
       <c r="F2" t="n">
-        <v>116036889</v>
+        <v>1.00611</v>
       </c>
       <c r="G2" t="n">
-        <v>116139029</v>
+        <v>5</v>
       </c>
       <c r="H2" t="n">
-        <v>10</v>
+        <v>87889197</v>
+      </c>
+      <c r="I2" t="n">
+        <v>88215594</v>
+      </c>
+      <c r="J2" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HC1007_TTE_acute_upper_respiratory_infections_of_multiple_and_unspecified_sites</t>
+          <t>HC219_Hypothyroidism/myxoedema</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>9q21.32</t>
+          <t>6p22.1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>AFR</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.26517 - (1.17674, 1.36024)</t>
+          <t>1.13952 (1.0892, 1.19217)</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1.98913e-10</v>
+        <v>1.44958e-08</v>
       </c>
       <c r="F3" t="n">
-        <v>85752837</v>
+        <v>0.977708</v>
       </c>
       <c r="G3" t="n">
-        <v>85810910</v>
+        <v>6</v>
       </c>
       <c r="H3" t="n">
-        <v>9</v>
+        <v>27312078</v>
+      </c>
+      <c r="I3" t="n">
+        <v>27491299</v>
+      </c>
+      <c r="J3" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HC643_TTE_other_hypothyroidism</t>
+          <t>HC326_Heart_attack_(MI)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6p21.33</t>
+          <t>5q14.3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>WAS</t>
+          <t>AFR</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.10766 - (1.07559, 1.14068)</t>
+          <t>0.531008 (0.417665, 0.675108)</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>9.041000000000001e-12</v>
+        <v>2.37668e-07</v>
       </c>
       <c r="F4" t="n">
-        <v>31428169</v>
+        <v>1.00647</v>
       </c>
       <c r="G4" t="n">
-        <v>31435326</v>
+        <v>5</v>
       </c>
       <c r="H4" t="n">
+        <v>87889197</v>
+      </c>
+      <c r="I4" t="n">
+        <v>88215594</v>
+      </c>
+      <c r="J4" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HC1581_AD_asthma</t>
+          <t>HC1158_TTE_other_dermatitis</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6p21.32</t>
+          <t>17p13.1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SAS</t>
+          <t>EAS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.911931 - (0.885, 0.939682)</t>
+          <t>1.41439 (1.23885, 1.6148)</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1.6632e-09</v>
+        <v>2.92945e-07</v>
       </c>
       <c r="F5" t="n">
-        <v>32207393</v>
+        <v>1.06558</v>
       </c>
       <c r="G5" t="n">
-        <v>32288190</v>
+        <v>17</v>
       </c>
       <c r="H5" t="n">
-        <v>6</v>
+        <v>8967469</v>
+      </c>
+      <c r="I5" t="n">
+        <v>9074101</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HC221_Diabetes</t>
+          <t>HC1036_TTE_asthma</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>8q24.13</t>
+          <t>6p21.33</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>SAS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.30723 - (1.20257, 1.421)</t>
+          <t>0.917315 (0.891119, 0.94428)</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3.12662e-10</v>
+        <v>5.26827e-09</v>
       </c>
       <c r="F6" t="n">
-        <v>124070432</v>
+        <v>1.09599</v>
       </c>
       <c r="G6" t="n">
-        <v>124092625</v>
+        <v>6</v>
       </c>
       <c r="H6" t="n">
-        <v>8</v>
+        <v>31461089</v>
+      </c>
+      <c r="I6" t="n">
+        <v>31465795</v>
+      </c>
+      <c r="J6" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HC382_Asthma</t>
+          <t>HC1581_AD_asthma</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>6p21.33</t>
+          <t>6p21.32</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>SAS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.952102 - (0.937014, 0.967432)</t>
+          <t>0.912836 (0.88496, 0.94159)</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>1.71636e-09</v>
+        <v>8.24137e-09</v>
       </c>
       <c r="F7" t="n">
-        <v>31346445</v>
+        <v>1.07725</v>
       </c>
       <c r="G7" t="n">
-        <v>31377047</v>
+        <v>6</v>
       </c>
       <c r="H7" t="n">
-        <v>6</v>
+        <v>32207393</v>
+      </c>
+      <c r="I7" t="n">
+        <v>32288190</v>
+      </c>
+      <c r="J7" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HC1581_AD_asthma</t>
+          <t>HC382_Asthma</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -687,36 +733,42 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>SAS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.952029 - (0.936851, 0.967452)</t>
+          <t>0.915912 (0.88972, 0.942874)</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2.02811e-09</v>
+        <v>2.96221e-09</v>
       </c>
       <c r="F8" t="n">
-        <v>31346445</v>
+        <v>1.0848</v>
       </c>
       <c r="G8" t="n">
-        <v>31377047</v>
+        <v>6</v>
       </c>
       <c r="H8" t="n">
-        <v>6</v>
+        <v>31461089</v>
+      </c>
+      <c r="I8" t="n">
+        <v>31465795</v>
+      </c>
+      <c r="J8" t="n">
+        <v>70</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>HC219_Hypothyroidism/myxoedema</t>
+          <t>HC164_Gastro-oesophageal_reflux_(gord)_/_gastric_reflux</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6p21.33</t>
+          <t>7p12.1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -726,26 +778,32 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.11714 - (1.08405, 1.15123)</t>
+          <t>1.15895 (1.0922, 1.22978)</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>5.16612e-13</v>
+        <v>1.09268e-06</v>
       </c>
       <c r="F9" t="n">
-        <v>31428169</v>
+        <v>0.947291</v>
       </c>
       <c r="G9" t="n">
-        <v>31435326</v>
+        <v>7</v>
       </c>
       <c r="H9" t="n">
-        <v>6</v>
+        <v>53177959</v>
+      </c>
+      <c r="I9" t="n">
+        <v>53340367</v>
+      </c>
+      <c r="J9" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>HC382_Asthma</t>
+          <t>HC219_Hypothyroidism/myxoedema</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -755,127 +813,71 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SAS</t>
+          <t>WAS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.913487 - (0.887258, 0.940491)</t>
+          <t>1.11719 (1.08332, 1.15212)</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>1.14581e-09</v>
+        <v>1.7196e-12</v>
       </c>
       <c r="F10" t="n">
-        <v>31905130</v>
+        <v>1.00575</v>
       </c>
       <c r="G10" t="n">
-        <v>32007956</v>
+        <v>6</v>
       </c>
       <c r="H10" t="n">
-        <v>6</v>
+        <v>31428169</v>
+      </c>
+      <c r="I10" t="n">
+        <v>31435326</v>
+      </c>
+      <c r="J10" t="n">
+        <v>58</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FH1220_Diabetes_(FH)</t>
+          <t>HC643_TTE_other_hypothyroidism</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>17p13.3</t>
+          <t>6p21.33</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>SAS</t>
+          <t>WAS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.21036 - (1.13851, 1.28675)</t>
+          <t>1.10308 (1.07039, 1.13677)</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>9.67926e-10</v>
+        <v>1.6432e-10</v>
       </c>
       <c r="F11" t="n">
-        <v>1820750</v>
+        <v>1.02831</v>
       </c>
       <c r="G11" t="n">
-        <v>1925859</v>
+        <v>6</v>
       </c>
       <c r="H11" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>HC1036_TTE_asthma</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>6p21.32</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>SAS</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>0.913471 - (0.886685, 0.941067)</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>2.52389e-09</v>
-      </c>
-      <c r="F12" t="n">
-        <v>32207393</v>
-      </c>
-      <c r="G12" t="n">
-        <v>32288190</v>
-      </c>
-      <c r="H12" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>HC221_Diabetes</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Timeout</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>1.23444 - (1.15216, 1.3226)</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>2.1687e-09</v>
-      </c>
-      <c r="F13" t="n">
-        <v>34958589</v>
-      </c>
-      <c r="G13" t="n">
-        <v>35158184</v>
-      </c>
-      <c r="H13" t="n">
-        <v>14</v>
+        <v>31428169</v>
+      </c>
+      <c r="I11" t="n">
+        <v>31435326</v>
+      </c>
+      <c r="J11" t="n">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>